<commit_message>
sync 2026-03-10 10:39 | precios/.~lock.lista_basicos.xlsx#,precios/lista_basicos.xlsx
</commit_message>
<xml_diff>
--- a/precios/lista_basicos.xlsx
+++ b/precios/lista_basicos.xlsx
@@ -8,7 +8,7 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId2"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -40,6 +40,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -59,19 +60,23 @@
     <font>
       <b val="true"/>
       <sz val="10"/>
+      <color rgb="FFEEEEEE"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FFEEEEEE"/>
       <name val="Inter"/>
       <family val="0"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="4">
@@ -128,21 +133,25 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -154,10 +163,40 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <dxfs count="4">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF3465A4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFEEEEEE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF2A6099"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
-      <rgbColor rgb="FFFFFFFF"/>
+      <rgbColor rgb="FFEEEEEE"/>
       <rgbColor rgb="FFFF0000"/>
       <rgbColor rgb="FF00FF00"/>
       <rgbColor rgb="FF0000FF"/>
@@ -217,112 +256,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office">
-  <a:themeElements>
-    <a:clrScheme name="LibreOffice">
-      <a:dk1>
-        <a:srgbClr val="000000"/>
-      </a:dk1>
-      <a:lt1>
-        <a:srgbClr val="ffffff"/>
-      </a:lt1>
-      <a:dk2>
-        <a:srgbClr val="000000"/>
-      </a:dk2>
-      <a:lt2>
-        <a:srgbClr val="ffffff"/>
-      </a:lt2>
-      <a:accent1>
-        <a:srgbClr val="18a303"/>
-      </a:accent1>
-      <a:accent2>
-        <a:srgbClr val="0369a3"/>
-      </a:accent2>
-      <a:accent3>
-        <a:srgbClr val="a33e03"/>
-      </a:accent3>
-      <a:accent4>
-        <a:srgbClr val="8e03a3"/>
-      </a:accent4>
-      <a:accent5>
-        <a:srgbClr val="c99c00"/>
-      </a:accent5>
-      <a:accent6>
-        <a:srgbClr val="c9211e"/>
-      </a:accent6>
-      <a:hlink>
-        <a:srgbClr val="0000ee"/>
-      </a:hlink>
-      <a:folHlink>
-        <a:srgbClr val="551a8b"/>
-      </a:folHlink>
-    </a:clrScheme>
-    <a:fontScheme name="Office">
-      <a:majorFont>
-        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
-        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
-        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
-      </a:majorFont>
-      <a:minorFont>
-        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
-        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
-        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
-      </a:minorFont>
-    </a:fontScheme>
-    <a:fmtScheme>
-      <a:fillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-      </a:fillStyleLst>
-      <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
-          <a:prstDash val="solid"/>
-          <a:miter/>
-        </a:ln>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
-          <a:prstDash val="solid"/>
-          <a:miter/>
-        </a:ln>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
-          <a:prstDash val="solid"/>
-          <a:miter/>
-        </a:ln>
-      </a:lnStyleLst>
-      <a:effectStyleLst>
-        <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-      </a:effectStyleLst>
-      <a:bgFillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-      </a:bgFillStyleLst>
-    </a:fmtScheme>
-  </a:themeElements>
-</a:theme>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
@@ -330,6 +263,9 @@
   </sheetPr>
   <dimension ref="A1:B206"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12.45"/>
+  </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -343,7 +279,7 @@
       <c r="A2" s="3" t="n">
         <v>1122608</v>
       </c>
-      <c r="B2" s="0" t="n">
+      <c r="B2" s="4" t="n">
         <v>360</v>
       </c>
     </row>
@@ -351,7 +287,7 @@
       <c r="A3" s="3" t="n">
         <v>1122605</v>
       </c>
-      <c r="B3" s="0" t="n">
+      <c r="B3" s="4" t="n">
         <v>360</v>
       </c>
     </row>
@@ -359,7 +295,7 @@
       <c r="A4" s="3" t="n">
         <v>1267023</v>
       </c>
-      <c r="B4" s="0" t="n">
+      <c r="B4" s="4" t="n">
         <v>360</v>
       </c>
     </row>
@@ -367,7 +303,7 @@
       <c r="A5" s="3" t="n">
         <v>1267022</v>
       </c>
-      <c r="B5" s="0" t="n">
+      <c r="B5" s="4" t="n">
         <v>360</v>
       </c>
     </row>
@@ -375,7 +311,7 @@
       <c r="A6" s="3" t="n">
         <v>1198171</v>
       </c>
-      <c r="B6" s="0" t="n">
+      <c r="B6" s="4" t="n">
         <v>360</v>
       </c>
     </row>
@@ -383,7 +319,7 @@
       <c r="A7" s="3" t="n">
         <v>1267026</v>
       </c>
-      <c r="B7" s="0" t="n">
+      <c r="B7" s="4" t="n">
         <v>380</v>
       </c>
     </row>
@@ -391,7 +327,7 @@
       <c r="A8" s="3" t="n">
         <v>1267025</v>
       </c>
-      <c r="B8" s="0" t="n">
+      <c r="B8" s="4" t="n">
         <v>380</v>
       </c>
     </row>
@@ -399,7 +335,7 @@
       <c r="A9" s="3" t="n">
         <v>1267167</v>
       </c>
-      <c r="B9" s="0" t="n">
+      <c r="B9" s="4" t="n">
         <v>470</v>
       </c>
     </row>
@@ -407,7 +343,7 @@
       <c r="A10" s="3" t="n">
         <v>1267168</v>
       </c>
-      <c r="B10" s="0" t="n">
+      <c r="B10" s="4" t="n">
         <v>470</v>
       </c>
     </row>
@@ -415,7 +351,7 @@
       <c r="A11" s="3" t="n">
         <v>1267164</v>
       </c>
-      <c r="B11" s="0" t="n">
+      <c r="B11" s="4" t="n">
         <v>400</v>
       </c>
     </row>
@@ -423,7 +359,7 @@
       <c r="A12" s="3" t="n">
         <v>1267165</v>
       </c>
-      <c r="B12" s="0" t="n">
+      <c r="B12" s="4" t="n">
         <v>400</v>
       </c>
     </row>
@@ -431,7 +367,7 @@
       <c r="A13" s="3" t="n">
         <v>1122613</v>
       </c>
-      <c r="B13" s="0" t="n">
+      <c r="B13" s="4" t="n">
         <v>360</v>
       </c>
     </row>
@@ -439,7 +375,7 @@
       <c r="A14" s="3" t="n">
         <v>1267024</v>
       </c>
-      <c r="B14" s="0" t="n">
+      <c r="B14" s="4" t="n">
         <v>360</v>
       </c>
     </row>
@@ -447,7 +383,7 @@
       <c r="A15" s="3" t="n">
         <v>1122615</v>
       </c>
-      <c r="B15" s="0" t="n">
+      <c r="B15" s="4" t="n">
         <v>360</v>
       </c>
     </row>
@@ -455,7 +391,7 @@
       <c r="A16" s="3" t="n">
         <v>1122614</v>
       </c>
-      <c r="B16" s="0" t="n">
+      <c r="B16" s="4" t="n">
         <v>360</v>
       </c>
     </row>
@@ -463,7 +399,7 @@
       <c r="A17" s="3" t="n">
         <v>1267169</v>
       </c>
-      <c r="B17" s="0" t="n">
+      <c r="B17" s="4" t="n">
         <v>400</v>
       </c>
     </row>
@@ -471,7 +407,7 @@
       <c r="A18" s="3" t="n">
         <v>1199184</v>
       </c>
-      <c r="B18" s="0" t="n">
+      <c r="B18" s="4" t="n">
         <v>400</v>
       </c>
     </row>
@@ -479,7 +415,7 @@
       <c r="A19" s="3" t="n">
         <v>1199183</v>
       </c>
-      <c r="B19" s="0" t="n">
+      <c r="B19" s="4" t="n">
         <v>400</v>
       </c>
     </row>
@@ -487,7 +423,7 @@
       <c r="A20" s="3" t="n">
         <v>1199182</v>
       </c>
-      <c r="B20" s="0" t="n">
+      <c r="B20" s="4" t="n">
         <v>400</v>
       </c>
     </row>
@@ -495,7 +431,7 @@
       <c r="A21" s="3" t="n">
         <v>1232289</v>
       </c>
-      <c r="B21" s="0" t="n">
+      <c r="B21" s="4" t="n">
         <v>410</v>
       </c>
     </row>
@@ -503,7 +439,7 @@
       <c r="A22" s="3" t="n">
         <v>1075951</v>
       </c>
-      <c r="B22" s="0" t="n">
+      <c r="B22" s="4" t="n">
         <v>410</v>
       </c>
     </row>
@@ -511,7 +447,7 @@
       <c r="A23" s="3" t="n">
         <v>1170207</v>
       </c>
-      <c r="B23" s="0" t="n">
+      <c r="B23" s="4" t="n">
         <v>380</v>
       </c>
     </row>
@@ -519,7 +455,7 @@
       <c r="A24" s="3" t="n">
         <v>1176821</v>
       </c>
-      <c r="B24" s="0" t="n">
+      <c r="B24" s="4" t="n">
         <v>410</v>
       </c>
     </row>
@@ -527,7 +463,7 @@
       <c r="A25" s="3" t="n">
         <v>1232290</v>
       </c>
-      <c r="B25" s="0" t="n">
+      <c r="B25" s="4" t="n">
         <v>410</v>
       </c>
     </row>
@@ -535,7 +471,7 @@
       <c r="A26" s="3" t="n">
         <v>1121183</v>
       </c>
-      <c r="B26" s="0" t="n">
+      <c r="B26" s="4" t="n">
         <v>410</v>
       </c>
     </row>
@@ -543,7 +479,7 @@
       <c r="A27" s="3" t="n">
         <v>1269535</v>
       </c>
-      <c r="B27" s="0" t="n">
+      <c r="B27" s="4" t="n">
         <v>440</v>
       </c>
     </row>
@@ -551,7 +487,7 @@
       <c r="A28" s="3" t="n">
         <v>1269531</v>
       </c>
-      <c r="B28" s="0" t="n">
+      <c r="B28" s="4" t="n">
         <v>380</v>
       </c>
     </row>
@@ -559,7 +495,7 @@
       <c r="A29" s="3" t="n">
         <v>1269530</v>
       </c>
-      <c r="B29" s="0" t="n">
+      <c r="B29" s="4" t="n">
         <v>380</v>
       </c>
     </row>
@@ -567,7 +503,7 @@
       <c r="A30" s="3" t="n">
         <v>1232285</v>
       </c>
-      <c r="B30" s="0" t="n">
+      <c r="B30" s="4" t="n">
         <v>450</v>
       </c>
     </row>
@@ -575,7 +511,7 @@
       <c r="A31" s="3" t="n">
         <v>1232286</v>
       </c>
-      <c r="B31" s="0" t="n">
+      <c r="B31" s="4" t="n">
         <v>440</v>
       </c>
     </row>
@@ -583,7 +519,7 @@
       <c r="A32" s="3" t="n">
         <v>1232287</v>
       </c>
-      <c r="B32" s="0" t="n">
+      <c r="B32" s="4" t="n">
         <v>440</v>
       </c>
     </row>
@@ -591,7 +527,7 @@
       <c r="A33" s="3" t="n">
         <v>1269528</v>
       </c>
-      <c r="B33" s="0" t="n">
+      <c r="B33" s="4" t="n">
         <v>510</v>
       </c>
     </row>
@@ -599,7 +535,7 @@
       <c r="A34" s="3" t="n">
         <v>1269527</v>
       </c>
-      <c r="B34" s="0" t="n">
+      <c r="B34" s="4" t="n">
         <v>510</v>
       </c>
     </row>
@@ -607,7 +543,7 @@
       <c r="A35" s="3" t="n">
         <v>1269526</v>
       </c>
-      <c r="B35" s="0" t="n">
+      <c r="B35" s="4" t="n">
         <v>470</v>
       </c>
     </row>
@@ -615,7 +551,7 @@
       <c r="A36" s="3" t="n">
         <v>1031514</v>
       </c>
-      <c r="B36" s="0" t="n">
+      <c r="B36" s="4" t="n">
         <v>470</v>
       </c>
     </row>
@@ -623,7 +559,7 @@
       <c r="A37" s="3" t="n">
         <v>1031465</v>
       </c>
-      <c r="B37" s="0" t="n">
+      <c r="B37" s="4" t="n">
         <v>470</v>
       </c>
     </row>
@@ -631,7 +567,7 @@
       <c r="A38" s="3" t="n">
         <v>1269532</v>
       </c>
-      <c r="B38" s="0" t="n">
+      <c r="B38" s="4" t="n">
         <v>470</v>
       </c>
     </row>
@@ -639,7 +575,7 @@
       <c r="A39" s="3" t="n">
         <v>1269533</v>
       </c>
-      <c r="B39" s="0" t="n">
+      <c r="B39" s="4" t="n">
         <v>470</v>
       </c>
     </row>
@@ -647,7 +583,7 @@
       <c r="A40" s="3" t="n">
         <v>1271740</v>
       </c>
-      <c r="B40" s="0" t="n">
+      <c r="B40" s="4" t="n">
         <v>470</v>
       </c>
     </row>
@@ -655,7 +591,7 @@
       <c r="A41" s="3" t="n">
         <v>1267166</v>
       </c>
-      <c r="B41" s="0" t="n">
+      <c r="B41" s="4" t="n">
         <v>470</v>
       </c>
     </row>
@@ -663,7 +599,7 @@
       <c r="A42" s="3" t="n">
         <v>1271741</v>
       </c>
-      <c r="B42" s="0" t="n">
+      <c r="B42" s="4" t="n">
         <v>470</v>
       </c>
     </row>
@@ -671,7 +607,7 @@
       <c r="A43" s="3" t="n">
         <v>989164</v>
       </c>
-      <c r="B43" s="0" t="n">
+      <c r="B43" s="4" t="n">
         <v>380</v>
       </c>
     </row>
@@ -679,7 +615,7 @@
       <c r="A44" s="3" t="n">
         <v>1269536</v>
       </c>
-      <c r="B44" s="0" t="n">
+      <c r="B44" s="4" t="n">
         <v>510</v>
       </c>
     </row>
@@ -687,7 +623,7 @@
       <c r="A45" s="3" t="n">
         <v>1279988</v>
       </c>
-      <c r="B45" s="0" t="n">
+      <c r="B45" s="4" t="n">
         <v>490</v>
       </c>
     </row>
@@ -695,7 +631,7 @@
       <c r="A46" s="3" t="n">
         <v>1267514</v>
       </c>
-      <c r="B46" s="0" t="n">
+      <c r="B46" s="4" t="n">
         <v>380</v>
       </c>
     </row>
@@ -703,7 +639,7 @@
       <c r="A47" s="3" t="n">
         <v>1267513</v>
       </c>
-      <c r="B47" s="0" t="n">
+      <c r="B47" s="4" t="n">
         <v>380</v>
       </c>
     </row>
@@ -711,7 +647,7 @@
       <c r="A48" s="3" t="n">
         <v>1119636</v>
       </c>
-      <c r="B48" s="0" t="n">
+      <c r="B48" s="4" t="n">
         <v>410</v>
       </c>
     </row>
@@ -719,7 +655,7 @@
       <c r="A49" s="3" t="n">
         <v>1267511</v>
       </c>
-      <c r="B49" s="0" t="n">
+      <c r="B49" s="4" t="n">
         <v>410</v>
       </c>
     </row>
@@ -727,7 +663,7 @@
       <c r="A50" s="3" t="n">
         <v>1267512</v>
       </c>
-      <c r="B50" s="0" t="n">
+      <c r="B50" s="4" t="n">
         <v>410</v>
       </c>
     </row>
@@ -735,7 +671,7 @@
       <c r="A51" s="3" t="n">
         <v>947788</v>
       </c>
-      <c r="B51" s="0" t="n">
+      <c r="B51" s="4" t="n">
         <v>490</v>
       </c>
     </row>
@@ -743,7 +679,7 @@
       <c r="A52" s="3" t="n">
         <v>1234264</v>
       </c>
-      <c r="B52" s="0" t="n">
+      <c r="B52" s="4" t="n">
         <v>490</v>
       </c>
     </row>
@@ -751,7 +687,7 @@
       <c r="A53" s="3" t="n">
         <v>947787</v>
       </c>
-      <c r="B53" s="0" t="n">
+      <c r="B53" s="4" t="n">
         <v>490</v>
       </c>
     </row>
@@ -759,7 +695,7 @@
       <c r="A54" s="3" t="n">
         <v>1268143</v>
       </c>
-      <c r="B54" s="0" t="n">
+      <c r="B54" s="4" t="n">
         <v>470</v>
       </c>
     </row>
@@ -767,7 +703,7 @@
       <c r="A55" s="3" t="n">
         <v>1199157</v>
       </c>
-      <c r="B55" s="0" t="n">
+      <c r="B55" s="4" t="n">
         <v>340</v>
       </c>
     </row>
@@ -775,7 +711,7 @@
       <c r="A56" s="3" t="n">
         <v>1017929</v>
       </c>
-      <c r="B56" s="0" t="n">
+      <c r="B56" s="4" t="n">
         <v>340</v>
       </c>
     </row>
@@ -783,7 +719,7 @@
       <c r="A57" s="3" t="n">
         <v>1017928</v>
       </c>
-      <c r="B57" s="0" t="n">
+      <c r="B57" s="4" t="n">
         <v>340</v>
       </c>
     </row>
@@ -791,7 +727,7 @@
       <c r="A58" s="3" t="n">
         <v>1283727</v>
       </c>
-      <c r="B58" s="0" t="n">
+      <c r="B58" s="4" t="n">
         <v>340</v>
       </c>
     </row>
@@ -799,7 +735,7 @@
       <c r="A59" s="3" t="n">
         <v>1267517</v>
       </c>
-      <c r="B59" s="0" t="n">
+      <c r="B59" s="4" t="n">
         <v>340</v>
       </c>
     </row>
@@ -807,7 +743,7 @@
       <c r="A60" s="3" t="n">
         <v>988231</v>
       </c>
-      <c r="B60" s="0" t="n">
+      <c r="B60" s="4" t="n">
         <v>340</v>
       </c>
     </row>
@@ -815,7 +751,7 @@
       <c r="A61" s="3" t="n">
         <v>988229</v>
       </c>
-      <c r="B61" s="0" t="n">
+      <c r="B61" s="4" t="n">
         <v>340</v>
       </c>
     </row>
@@ -823,7 +759,7 @@
       <c r="A62" s="3" t="n">
         <v>1267516</v>
       </c>
-      <c r="B62" s="0" t="n">
+      <c r="B62" s="4" t="n">
         <v>380</v>
       </c>
     </row>
@@ -831,7 +767,7 @@
       <c r="A63" s="3" t="n">
         <v>176593</v>
       </c>
-      <c r="B63" s="0" t="n">
+      <c r="B63" s="4" t="n">
         <v>380</v>
       </c>
     </row>
@@ -839,7 +775,7 @@
       <c r="A64" s="3" t="n">
         <v>166303</v>
       </c>
-      <c r="B64" s="0" t="n">
+      <c r="B64" s="4" t="n">
         <v>380</v>
       </c>
     </row>
@@ -847,7 +783,7 @@
       <c r="A65" s="3" t="n">
         <v>143138</v>
       </c>
-      <c r="B65" s="0" t="n">
+      <c r="B65" s="4" t="n">
         <v>400</v>
       </c>
     </row>
@@ -855,7 +791,7 @@
       <c r="A66" s="3" t="n">
         <v>133241</v>
       </c>
-      <c r="B66" s="0" t="n">
+      <c r="B66" s="4" t="n">
         <v>380</v>
       </c>
     </row>
@@ -863,7 +799,7 @@
       <c r="A67" s="3" t="n">
         <v>133240</v>
       </c>
-      <c r="B67" s="0" t="n">
+      <c r="B67" s="4" t="n">
         <v>400</v>
       </c>
     </row>
@@ -871,7 +807,7 @@
       <c r="A68" s="3" t="n">
         <v>1267515</v>
       </c>
-      <c r="B68" s="0" t="n">
+      <c r="B68" s="4" t="n">
         <v>380</v>
       </c>
     </row>
@@ -879,7 +815,7 @@
       <c r="A69" s="3" t="n">
         <v>176588</v>
       </c>
-      <c r="B69" s="0" t="n">
+      <c r="B69" s="4" t="n">
         <v>380</v>
       </c>
     </row>
@@ -887,7 +823,7 @@
       <c r="A70" s="3" t="n">
         <v>133256</v>
       </c>
-      <c r="B70" s="0" t="n">
+      <c r="B70" s="4" t="n">
         <v>400</v>
       </c>
     </row>
@@ -895,7 +831,7 @@
       <c r="A71" s="3" t="n">
         <v>133254</v>
       </c>
-      <c r="B71" s="0" t="n">
+      <c r="B71" s="4" t="n">
         <v>380</v>
       </c>
     </row>
@@ -903,7 +839,7 @@
       <c r="A72" s="3" t="n">
         <v>133251</v>
       </c>
-      <c r="B72" s="0" t="n">
+      <c r="B72" s="4" t="n">
         <v>400</v>
       </c>
     </row>
@@ -911,7 +847,7 @@
       <c r="A73" s="3" t="n">
         <v>133250</v>
       </c>
-      <c r="B73" s="0" t="n">
+      <c r="B73" s="4" t="n">
         <v>400</v>
       </c>
     </row>
@@ -919,7 +855,7 @@
       <c r="A74" s="3" t="n">
         <v>1182056</v>
       </c>
-      <c r="B74" s="0" t="n">
+      <c r="B74" s="4" t="n">
         <v>380</v>
       </c>
     </row>
@@ -927,7 +863,7 @@
       <c r="A75" s="3" t="n">
         <v>831147</v>
       </c>
-      <c r="B75" s="0" t="n">
+      <c r="B75" s="4" t="n">
         <v>380</v>
       </c>
     </row>
@@ -935,7 +871,7 @@
       <c r="A76" s="3" t="n">
         <v>1228140</v>
       </c>
-      <c r="B76" s="0" t="n">
+      <c r="B76" s="4" t="n">
         <v>380</v>
       </c>
     </row>
@@ -943,7 +879,7 @@
       <c r="A77" s="3" t="n">
         <v>1226315</v>
       </c>
-      <c r="B77" s="0" t="n">
+      <c r="B77" s="4" t="n">
         <v>340</v>
       </c>
     </row>
@@ -951,7 +887,7 @@
       <c r="A78" s="3" t="n">
         <v>1228143</v>
       </c>
-      <c r="B78" s="0" t="n">
+      <c r="B78" s="4" t="n">
         <v>380</v>
       </c>
     </row>
@@ -959,7 +895,7 @@
       <c r="A79" s="3" t="n">
         <v>1228142</v>
       </c>
-      <c r="B79" s="0" t="n">
+      <c r="B79" s="4" t="n">
         <v>360</v>
       </c>
     </row>
@@ -967,7 +903,7 @@
       <c r="A80" s="3" t="n">
         <v>1267176</v>
       </c>
-      <c r="B80" s="0" t="n">
+      <c r="B80" s="4" t="n">
         <v>380</v>
       </c>
     </row>
@@ -975,7 +911,7 @@
       <c r="A81" s="3" t="n">
         <v>1267175</v>
       </c>
-      <c r="B81" s="0" t="n">
+      <c r="B81" s="4" t="n">
         <v>380</v>
       </c>
     </row>
@@ -983,7 +919,7 @@
       <c r="A82" s="3" t="n">
         <v>1267173</v>
       </c>
-      <c r="B82" s="0" t="n">
+      <c r="B82" s="4" t="n">
         <v>380</v>
       </c>
     </row>
@@ -991,7 +927,7 @@
       <c r="A83" s="3" t="n">
         <v>1267171</v>
       </c>
-      <c r="B83" s="0" t="n">
+      <c r="B83" s="4" t="n">
         <v>380</v>
       </c>
     </row>
@@ -999,7 +935,7 @@
       <c r="A84" s="3" t="n">
         <v>1267170</v>
       </c>
-      <c r="B84" s="0" t="n">
+      <c r="B84" s="4" t="n">
         <v>380</v>
       </c>
     </row>
@@ -1007,7 +943,7 @@
       <c r="A85" s="3" t="n">
         <v>1267178</v>
       </c>
-      <c r="B85" s="0" t="n">
+      <c r="B85" s="4" t="n">
         <v>380</v>
       </c>
     </row>
@@ -1015,7 +951,7 @@
       <c r="A86" s="3" t="n">
         <v>1267174</v>
       </c>
-      <c r="B86" s="0" t="n">
+      <c r="B86" s="4" t="n">
         <v>380</v>
       </c>
     </row>
@@ -1023,7 +959,7 @@
       <c r="A87" s="3" t="n">
         <v>1267172</v>
       </c>
-      <c r="B87" s="0" t="n">
+      <c r="B87" s="4" t="n">
         <v>380</v>
       </c>
     </row>
@@ -1031,7 +967,7 @@
       <c r="A88" s="3" t="n">
         <v>1267030</v>
       </c>
-      <c r="B88" s="0" t="n">
+      <c r="B88" s="4" t="n">
         <v>450</v>
       </c>
     </row>
@@ -1039,7 +975,7 @@
       <c r="A89" s="3" t="n">
         <v>1267029</v>
       </c>
-      <c r="B89" s="0" t="n">
+      <c r="B89" s="4" t="n">
         <v>450</v>
       </c>
     </row>
@@ -1047,7 +983,7 @@
       <c r="A90" s="3" t="n">
         <v>1267028</v>
       </c>
-      <c r="B90" s="0" t="n">
+      <c r="B90" s="4" t="n">
         <v>470</v>
       </c>
     </row>
@@ -1055,7 +991,7 @@
       <c r="A91" s="3" t="n">
         <v>1267027</v>
       </c>
-      <c r="B91" s="0" t="n">
+      <c r="B91" s="4" t="n">
         <v>470</v>
       </c>
     </row>
@@ -1063,7 +999,7 @@
       <c r="A92" s="3" t="n">
         <v>1269538</v>
       </c>
-      <c r="B92" s="0" t="n">
+      <c r="B92" s="4" t="n">
         <v>520</v>
       </c>
     </row>
@@ -1071,7 +1007,7 @@
       <c r="A93" s="3" t="n">
         <v>1269539</v>
       </c>
-      <c r="B93" s="0" t="n">
+      <c r="B93" s="4" t="n">
         <v>520</v>
       </c>
     </row>
@@ -1079,7 +1015,7 @@
       <c r="A94" s="3" t="n">
         <v>1269537</v>
       </c>
-      <c r="B94" s="0" t="n">
+      <c r="B94" s="4" t="n">
         <v>520</v>
       </c>
     </row>
@@ -1087,7 +1023,7 @@
       <c r="A95" s="3" t="n">
         <v>1214911</v>
       </c>
-      <c r="B95" s="0" t="n">
+      <c r="B95" s="4" t="n">
         <v>520</v>
       </c>
     </row>
@@ -1095,7 +1031,7 @@
       <c r="A96" s="3" t="n">
         <v>1214910</v>
       </c>
-      <c r="B96" s="0" t="n">
+      <c r="B96" s="4" t="n">
         <v>520</v>
       </c>
     </row>
@@ -1103,7 +1039,7 @@
       <c r="A97" s="3" t="n">
         <v>1269542</v>
       </c>
-      <c r="B97" s="0" t="n">
+      <c r="B97" s="4" t="n">
         <v>420</v>
       </c>
     </row>
@@ -1111,7 +1047,7 @@
       <c r="A98" s="3" t="n">
         <v>1269541</v>
       </c>
-      <c r="B98" s="0" t="n">
+      <c r="B98" s="4" t="n">
         <v>440</v>
       </c>
     </row>
@@ -1119,7 +1055,7 @@
       <c r="A99" s="3" t="n">
         <v>1269540</v>
       </c>
-      <c r="B99" s="0" t="n">
+      <c r="B99" s="4" t="n">
         <v>420</v>
       </c>
     </row>
@@ -1127,7 +1063,7 @@
       <c r="A100" s="3" t="n">
         <v>1214267</v>
       </c>
-      <c r="B100" s="0" t="n">
+      <c r="B100" s="4" t="n">
         <v>440</v>
       </c>
     </row>
@@ -1135,7 +1071,7 @@
       <c r="A101" s="3" t="n">
         <v>1011086</v>
       </c>
-      <c r="B101" s="0" t="n">
+      <c r="B101" s="4" t="n">
         <v>260</v>
       </c>
     </row>
@@ -1143,7 +1079,7 @@
       <c r="A102" s="3" t="n">
         <v>1004183</v>
       </c>
-      <c r="B102" s="0" t="n">
+      <c r="B102" s="4" t="n">
         <v>260</v>
       </c>
     </row>
@@ -1151,7 +1087,7 @@
       <c r="A103" s="3" t="n">
         <v>1004182</v>
       </c>
-      <c r="B103" s="0" t="n">
+      <c r="B103" s="4" t="n">
         <v>260</v>
       </c>
     </row>
@@ -1159,7 +1095,7 @@
       <c r="A104" s="3" t="n">
         <v>1286088</v>
       </c>
-      <c r="B104" s="0" t="n">
+      <c r="B104" s="4" t="n">
         <v>400</v>
       </c>
     </row>
@@ -1167,7 +1103,7 @@
       <c r="A105" s="3" t="n">
         <v>1286087</v>
       </c>
-      <c r="B105" s="0" t="n">
+      <c r="B105" s="4" t="n">
         <v>400</v>
       </c>
     </row>
@@ -1175,7 +1111,7 @@
       <c r="A106" s="3" t="n">
         <v>1286086</v>
       </c>
-      <c r="B106" s="0" t="n">
+      <c r="B106" s="4" t="n">
         <v>400</v>
       </c>
     </row>
@@ -1183,7 +1119,7 @@
       <c r="A107" s="3" t="n">
         <v>1286085</v>
       </c>
-      <c r="B107" s="0" t="n">
+      <c r="B107" s="4" t="n">
         <v>400</v>
       </c>
     </row>
@@ -1191,7 +1127,7 @@
       <c r="A108" s="3" t="n">
         <v>1128489</v>
       </c>
-      <c r="B108" s="0" t="n">
+      <c r="B108" s="4" t="n">
         <v>380</v>
       </c>
     </row>
@@ -1199,7 +1135,7 @@
       <c r="A109" s="3" t="n">
         <v>1081690</v>
       </c>
-      <c r="B109" s="0" t="n">
+      <c r="B109" s="4" t="n">
         <v>400</v>
       </c>
     </row>
@@ -1207,7 +1143,7 @@
       <c r="A110" s="3" t="n">
         <v>1081689</v>
       </c>
-      <c r="B110" s="0" t="n">
+      <c r="B110" s="4" t="n">
         <v>400</v>
       </c>
     </row>
@@ -1215,7 +1151,7 @@
       <c r="A111" s="3" t="n">
         <v>1202168</v>
       </c>
-      <c r="B111" s="0" t="n">
+      <c r="B111" s="4" t="n">
         <v>360</v>
       </c>
     </row>
@@ -1223,7 +1159,7 @@
       <c r="A112" s="3" t="n">
         <v>1004181</v>
       </c>
-      <c r="B112" s="0" t="n">
+      <c r="B112" s="4" t="n">
         <v>360</v>
       </c>
     </row>
@@ -1231,7 +1167,7 @@
       <c r="A113" s="3" t="n">
         <v>1004178</v>
       </c>
-      <c r="B113" s="0" t="n">
+      <c r="B113" s="4" t="n">
         <v>360</v>
       </c>
     </row>
@@ -1239,7 +1175,7 @@
       <c r="A114" s="3" t="n">
         <v>1286081</v>
       </c>
-      <c r="B114" s="0" t="n">
+      <c r="B114" s="4" t="n">
         <v>360</v>
       </c>
     </row>
@@ -1247,7 +1183,7 @@
       <c r="A115" s="3" t="n">
         <v>1286080</v>
       </c>
-      <c r="B115" s="0" t="n">
+      <c r="B115" s="4" t="n">
         <v>360</v>
       </c>
     </row>
@@ -1255,7 +1191,7 @@
       <c r="A116" s="3" t="n">
         <v>1241779</v>
       </c>
-      <c r="B116" s="0" t="n">
+      <c r="B116" s="4" t="n">
         <v>400</v>
       </c>
     </row>
@@ -1263,7 +1199,7 @@
       <c r="A117" s="3" t="n">
         <v>1004188</v>
       </c>
-      <c r="B117" s="0" t="n">
+      <c r="B117" s="4" t="n">
         <v>380</v>
       </c>
     </row>
@@ -1271,7 +1207,7 @@
       <c r="A118" s="3" t="n">
         <v>1004187</v>
       </c>
-      <c r="B118" s="0" t="n">
+      <c r="B118" s="4" t="n">
         <v>380</v>
       </c>
     </row>
@@ -1279,7 +1215,7 @@
       <c r="A119" s="3" t="n">
         <v>1241789</v>
       </c>
-      <c r="B119" s="0" t="n">
+      <c r="B119" s="4" t="n">
         <v>260</v>
       </c>
     </row>
@@ -1287,7 +1223,7 @@
       <c r="A120" s="3" t="n">
         <v>1286083</v>
       </c>
-      <c r="B120" s="0" t="n">
+      <c r="B120" s="4" t="n">
         <v>380</v>
       </c>
     </row>
@@ -1295,7 +1231,7 @@
       <c r="A121" s="3" t="n">
         <v>1241782</v>
       </c>
-      <c r="B121" s="0" t="n">
+      <c r="B121" s="4" t="n">
         <v>400</v>
       </c>
     </row>
@@ -1303,7 +1239,7 @@
       <c r="A122" s="3" t="n">
         <v>1241781</v>
       </c>
-      <c r="B122" s="0" t="n">
+      <c r="B122" s="4" t="n">
         <v>400</v>
       </c>
     </row>
@@ -1311,7 +1247,7 @@
       <c r="A123" s="3" t="n">
         <v>1081687</v>
       </c>
-      <c r="B123" s="0" t="n">
+      <c r="B123" s="4" t="n">
         <v>380</v>
       </c>
     </row>
@@ -1319,7 +1255,7 @@
       <c r="A124" s="3" t="n">
         <v>1081686</v>
       </c>
-      <c r="B124" s="0" t="n">
+      <c r="B124" s="4" t="n">
         <v>380</v>
       </c>
     </row>
@@ -1327,7 +1263,7 @@
       <c r="A125" s="3" t="n">
         <v>1286084</v>
       </c>
-      <c r="B125" s="0" t="n">
+      <c r="B125" s="4" t="n">
         <v>380</v>
       </c>
     </row>
@@ -1335,7 +1271,7 @@
       <c r="A126" s="3" t="n">
         <v>1286095</v>
       </c>
-      <c r="B126" s="0" t="n">
+      <c r="B126" s="4" t="n">
         <v>260</v>
       </c>
     </row>
@@ -1343,7 +1279,7 @@
       <c r="A127" s="3" t="n">
         <v>1286096</v>
       </c>
-      <c r="B127" s="0" t="n">
+      <c r="B127" s="4" t="n">
         <v>260</v>
       </c>
     </row>
@@ -1351,7 +1287,7 @@
       <c r="A128" s="3" t="n">
         <v>1286094</v>
       </c>
-      <c r="B128" s="0" t="n">
+      <c r="B128" s="4" t="n">
         <v>260</v>
       </c>
     </row>
@@ -1359,7 +1295,7 @@
       <c r="A129" s="3" t="n">
         <v>1286093</v>
       </c>
-      <c r="B129" s="0" t="n">
+      <c r="B129" s="4" t="n">
         <v>260</v>
       </c>
     </row>
@@ -1367,7 +1303,7 @@
       <c r="A130" s="3" t="n">
         <v>1286092</v>
       </c>
-      <c r="B130" s="0" t="n">
+      <c r="B130" s="4" t="n">
         <v>260</v>
       </c>
     </row>
@@ -1375,7 +1311,7 @@
       <c r="A131" s="3" t="n">
         <v>1065071</v>
       </c>
-      <c r="B131" s="0" t="n">
+      <c r="B131" s="4" t="n">
         <v>440</v>
       </c>
     </row>
@@ -1383,7 +1319,7 @@
       <c r="A132" s="3" t="n">
         <v>183774</v>
       </c>
-      <c r="B132" s="0" t="n">
+      <c r="B132" s="4" t="n">
         <v>440</v>
       </c>
     </row>
@@ -1391,7 +1327,7 @@
       <c r="A133" s="3" t="n">
         <v>831160</v>
       </c>
-      <c r="B133" s="0" t="n">
+      <c r="B133" s="4" t="n">
         <v>470</v>
       </c>
     </row>
@@ -1399,7 +1335,7 @@
       <c r="A134" s="3" t="n">
         <v>1268141</v>
       </c>
-      <c r="B134" s="0" t="n">
+      <c r="B134" s="4" t="n">
         <v>690</v>
       </c>
     </row>
@@ -1407,7 +1343,7 @@
       <c r="A135" s="3" t="n">
         <v>1268142</v>
       </c>
-      <c r="B135" s="0" t="n">
+      <c r="B135" s="4" t="n">
         <v>700</v>
       </c>
     </row>
@@ -1415,7 +1351,7 @@
       <c r="A136" s="3" t="n">
         <v>162170</v>
       </c>
-      <c r="B136" s="0" t="n">
+      <c r="B136" s="4" t="n">
         <v>1050</v>
       </c>
     </row>
@@ -1423,7 +1359,7 @@
       <c r="A137" s="3" t="n">
         <v>1066969</v>
       </c>
-      <c r="B137" s="0" t="n">
+      <c r="B137" s="4" t="n">
         <v>520</v>
       </c>
     </row>
@@ -1431,7 +1367,7 @@
       <c r="A138" s="3" t="n">
         <v>1066967</v>
       </c>
-      <c r="B138" s="0" t="n">
+      <c r="B138" s="4" t="n">
         <v>520</v>
       </c>
     </row>
@@ -1439,7 +1375,7 @@
       <c r="A139" s="3" t="n">
         <v>1066966</v>
       </c>
-      <c r="B139" s="0" t="n">
+      <c r="B139" s="4" t="n">
         <v>520</v>
       </c>
     </row>
@@ -1447,7 +1383,7 @@
       <c r="A140" s="3" t="n">
         <v>1032629</v>
       </c>
-      <c r="B140" s="0" t="n">
+      <c r="B140" s="4" t="n">
         <v>520</v>
       </c>
     </row>
@@ -1455,7 +1391,7 @@
       <c r="A141" s="3" t="n">
         <v>1032627</v>
       </c>
-      <c r="B141" s="0" t="n">
+      <c r="B141" s="4" t="n">
         <v>520</v>
       </c>
     </row>
@@ -1463,7 +1399,7 @@
       <c r="A142" s="3" t="n">
         <v>1032624</v>
       </c>
-      <c r="B142" s="0" t="n">
+      <c r="B142" s="4" t="n">
         <v>520</v>
       </c>
     </row>
@@ -1471,7 +1407,7 @@
       <c r="A143" s="3" t="n">
         <v>1032623</v>
       </c>
-      <c r="B143" s="0" t="n">
+      <c r="B143" s="4" t="n">
         <v>520</v>
       </c>
     </row>
@@ -1479,7 +1415,7 @@
       <c r="A144" s="3" t="n">
         <v>173544</v>
       </c>
-      <c r="B144" s="0" t="n">
+      <c r="B144" s="4" t="n">
         <v>760</v>
       </c>
     </row>
@@ -1487,7 +1423,7 @@
       <c r="A145" s="3" t="n">
         <v>173543</v>
       </c>
-      <c r="B145" s="0" t="n">
+      <c r="B145" s="4" t="n">
         <v>760</v>
       </c>
     </row>
@@ -1495,7 +1431,7 @@
       <c r="A146" s="3" t="n">
         <v>831113</v>
       </c>
-      <c r="B146" s="0" t="n">
+      <c r="B146" s="4" t="n">
         <v>760</v>
       </c>
     </row>
@@ -1503,7 +1439,7 @@
       <c r="A147" s="3" t="n">
         <v>823357</v>
       </c>
-      <c r="B147" s="0" t="n">
+      <c r="B147" s="4" t="n">
         <v>760</v>
       </c>
     </row>
@@ -1511,7 +1447,7 @@
       <c r="A148" s="3" t="n">
         <v>1226708</v>
       </c>
-      <c r="B148" s="0" t="n">
+      <c r="B148" s="4" t="n">
         <v>760</v>
       </c>
     </row>
@@ -1519,7 +1455,7 @@
       <c r="A149" s="3" t="n">
         <v>995373</v>
       </c>
-      <c r="B149" s="0" t="n">
+      <c r="B149" s="4" t="n">
         <v>760</v>
       </c>
     </row>
@@ -1527,7 +1463,7 @@
       <c r="A150" s="3" t="n">
         <v>985607</v>
       </c>
-      <c r="B150" s="0" t="n">
+      <c r="B150" s="4" t="n">
         <v>760</v>
       </c>
     </row>
@@ -1535,7 +1471,7 @@
       <c r="A151" s="3" t="n">
         <v>831295</v>
       </c>
-      <c r="B151" s="0" t="n">
+      <c r="B151" s="4" t="n">
         <v>760</v>
       </c>
     </row>
@@ -1543,7 +1479,7 @@
       <c r="A152" s="3" t="n">
         <v>1068769</v>
       </c>
-      <c r="B152" s="0" t="n">
+      <c r="B152" s="4" t="n">
         <v>760</v>
       </c>
     </row>
@@ -1551,7 +1487,7 @@
       <c r="A153" s="3" t="n">
         <v>1034973</v>
       </c>
-      <c r="B153" s="0" t="n">
+      <c r="B153" s="4" t="n">
         <v>760</v>
       </c>
     </row>
@@ -1559,7 +1495,7 @@
       <c r="A154" s="3" t="n">
         <v>1199208</v>
       </c>
-      <c r="B154" s="0" t="n">
+      <c r="B154" s="4" t="n">
         <v>660</v>
       </c>
     </row>
@@ -1567,7 +1503,7 @@
       <c r="A155" s="3" t="n">
         <v>1116409</v>
       </c>
-      <c r="B155" s="0" t="n">
+      <c r="B155" s="4" t="n">
         <v>830</v>
       </c>
     </row>
@@ -1575,7 +1511,7 @@
       <c r="A156" s="3" t="n">
         <v>1015337</v>
       </c>
-      <c r="B156" s="0" t="n">
+      <c r="B156" s="4" t="n">
         <v>400</v>
       </c>
     </row>
@@ -1583,7 +1519,7 @@
       <c r="A157" s="3" t="n">
         <v>1076549</v>
       </c>
-      <c r="B157" s="0" t="n">
+      <c r="B157" s="4" t="n">
         <v>650</v>
       </c>
     </row>
@@ -1591,7 +1527,7 @@
       <c r="A158" s="3" t="n">
         <v>155531</v>
       </c>
-      <c r="B158" s="0" t="n">
+      <c r="B158" s="4" t="n">
         <v>650</v>
       </c>
     </row>
@@ -1599,7 +1535,7 @@
       <c r="A159" s="3" t="n">
         <v>1076543</v>
       </c>
-      <c r="B159" s="0" t="n">
+      <c r="B159" s="4" t="n">
         <v>650</v>
       </c>
     </row>
@@ -1607,7 +1543,7 @@
       <c r="A160" s="3" t="n">
         <v>167317</v>
       </c>
-      <c r="B160" s="0" t="n">
+      <c r="B160" s="4" t="n">
         <v>650</v>
       </c>
     </row>
@@ -1615,7 +1551,7 @@
       <c r="A161" s="3" t="n">
         <v>144641</v>
       </c>
-      <c r="B161" s="0" t="n">
+      <c r="B161" s="4" t="n">
         <v>650</v>
       </c>
     </row>
@@ -1623,7 +1559,7 @@
       <c r="A162" s="3" t="n">
         <v>139918</v>
       </c>
-      <c r="B162" s="0" t="n">
+      <c r="B162" s="4" t="n">
         <v>650</v>
       </c>
     </row>
@@ -1631,7 +1567,7 @@
       <c r="A163" s="3" t="n">
         <v>1154597</v>
       </c>
-      <c r="B163" s="0" t="n">
+      <c r="B163" s="4" t="n">
         <v>650</v>
       </c>
     </row>
@@ -1639,7 +1575,7 @@
       <c r="A164" s="3" t="n">
         <v>1274315</v>
       </c>
-      <c r="B164" s="0" t="n">
+      <c r="B164" s="4" t="n">
         <v>510</v>
       </c>
     </row>
@@ -1647,7 +1583,7 @@
       <c r="A165" s="3" t="n">
         <v>1161871</v>
       </c>
-      <c r="B165" s="0" t="n">
+      <c r="B165" s="4" t="n">
         <v>510</v>
       </c>
     </row>
@@ -1655,7 +1591,7 @@
       <c r="A166" s="3" t="n">
         <v>1069621</v>
       </c>
-      <c r="B166" s="0" t="n">
+      <c r="B166" s="4" t="n">
         <v>510</v>
       </c>
     </row>
@@ -1663,7 +1599,7 @@
       <c r="A167" s="3" t="n">
         <v>1069619</v>
       </c>
-      <c r="B167" s="0" t="n">
+      <c r="B167" s="4" t="n">
         <v>510</v>
       </c>
     </row>
@@ -1671,7 +1607,7 @@
       <c r="A168" s="3" t="n">
         <v>1069618</v>
       </c>
-      <c r="B168" s="0" t="n">
+      <c r="B168" s="4" t="n">
         <v>510</v>
       </c>
     </row>
@@ -1679,7 +1615,7 @@
       <c r="A169" s="3" t="n">
         <v>166785</v>
       </c>
-      <c r="B169" s="0" t="n">
+      <c r="B169" s="4" t="n">
         <v>490</v>
       </c>
     </row>
@@ -1687,7 +1623,7 @@
       <c r="A170" s="3" t="n">
         <v>166173</v>
       </c>
-      <c r="B170" s="0" t="n">
+      <c r="B170" s="4" t="n">
         <v>490</v>
       </c>
     </row>
@@ -1695,7 +1631,7 @@
       <c r="A171" s="3" t="n">
         <v>166172</v>
       </c>
-      <c r="B171" s="0" t="n">
+      <c r="B171" s="4" t="n">
         <v>490</v>
       </c>
     </row>
@@ -1703,7 +1639,7 @@
       <c r="A172" s="3" t="n">
         <v>166159</v>
       </c>
-      <c r="B172" s="0" t="n">
+      <c r="B172" s="4" t="n">
         <v>490</v>
       </c>
     </row>
@@ -1711,7 +1647,7 @@
       <c r="A173" s="3" t="n">
         <v>907018</v>
       </c>
-      <c r="B173" s="0" t="n">
+      <c r="B173" s="4" t="n">
         <v>510</v>
       </c>
     </row>
@@ -1719,7 +1655,7 @@
       <c r="A174" s="3" t="n">
         <v>831813</v>
       </c>
-      <c r="B174" s="0" t="n">
+      <c r="B174" s="4" t="n">
         <v>510</v>
       </c>
     </row>
@@ -1727,7 +1663,7 @@
       <c r="A175" s="3" t="n">
         <v>183976</v>
       </c>
-      <c r="B175" s="0" t="n">
+      <c r="B175" s="4" t="n">
         <v>510</v>
       </c>
     </row>
@@ -1735,7 +1671,7 @@
       <c r="A176" s="3" t="n">
         <v>166809</v>
       </c>
-      <c r="B176" s="0" t="n">
+      <c r="B176" s="4" t="n">
         <v>440</v>
       </c>
     </row>
@@ -1743,7 +1679,7 @@
       <c r="A177" s="3" t="n">
         <v>996940</v>
       </c>
-      <c r="B177" s="0" t="n">
+      <c r="B177" s="4" t="n">
         <v>440</v>
       </c>
     </row>
@@ -1751,7 +1687,7 @@
       <c r="A178" s="3" t="n">
         <v>1022097</v>
       </c>
-      <c r="B178" s="0" t="n">
+      <c r="B178" s="4" t="n">
         <v>400</v>
       </c>
     </row>
@@ -1759,7 +1695,7 @@
       <c r="A179" s="3" t="n">
         <v>1202152</v>
       </c>
-      <c r="B179" s="0" t="n">
+      <c r="B179" s="4" t="n">
         <v>400</v>
       </c>
     </row>
@@ -1767,7 +1703,7 @@
       <c r="A180" s="3" t="n">
         <v>1071054</v>
       </c>
-      <c r="B180" s="0" t="n">
+      <c r="B180" s="4" t="n">
         <v>400</v>
       </c>
     </row>
@@ -1775,7 +1711,7 @@
       <c r="A181" s="3" t="n">
         <v>1202154</v>
       </c>
-      <c r="B181" s="0" t="n">
+      <c r="B181" s="4" t="n">
         <v>340</v>
       </c>
     </row>
@@ -1783,7 +1719,7 @@
       <c r="A182" s="3" t="n">
         <v>1132454</v>
       </c>
-      <c r="B182" s="0" t="n">
+      <c r="B182" s="4" t="n">
         <v>340</v>
       </c>
     </row>
@@ -1791,7 +1727,7 @@
       <c r="A183" s="3" t="n">
         <v>1271683</v>
       </c>
-      <c r="B183" s="0" t="n">
+      <c r="B183" s="4" t="n">
         <v>340</v>
       </c>
     </row>
@@ -1799,7 +1735,7 @@
       <c r="A184" s="3" t="n">
         <v>1158789</v>
       </c>
-      <c r="B184" s="0" t="n">
+      <c r="B184" s="4" t="n">
         <v>340</v>
       </c>
     </row>
@@ -1807,7 +1743,7 @@
       <c r="A185" s="3" t="n">
         <v>1132455</v>
       </c>
-      <c r="B185" s="0" t="n">
+      <c r="B185" s="4" t="n">
         <v>340</v>
       </c>
     </row>
@@ -1815,7 +1751,7 @@
       <c r="A186" s="3" t="n">
         <v>1232349</v>
       </c>
-      <c r="B186" s="0" t="n">
+      <c r="B186" s="4" t="n">
         <v>340</v>
       </c>
     </row>
@@ -1823,7 +1759,7 @@
       <c r="A187" s="3" t="n">
         <v>1202153</v>
       </c>
-      <c r="B187" s="0" t="n">
+      <c r="B187" s="4" t="n">
         <v>340</v>
       </c>
     </row>
@@ -1831,7 +1767,7 @@
       <c r="A188" s="3" t="n">
         <v>1017977</v>
       </c>
-      <c r="B188" s="0" t="n">
+      <c r="B188" s="4" t="n">
         <v>340</v>
       </c>
     </row>
@@ -1839,7 +1775,7 @@
       <c r="A189" s="3" t="n">
         <v>175929</v>
       </c>
-      <c r="B189" s="0" t="n">
+      <c r="B189" s="4" t="n">
         <v>340</v>
       </c>
     </row>
@@ -1847,7 +1783,7 @@
       <c r="A190" s="3" t="n">
         <v>121434</v>
       </c>
-      <c r="B190" s="0" t="n">
+      <c r="B190" s="4" t="n">
         <v>340</v>
       </c>
     </row>
@@ -1855,7 +1791,7 @@
       <c r="A191" s="3" t="n">
         <v>121432</v>
       </c>
-      <c r="B191" s="0" t="n">
+      <c r="B191" s="4" t="n">
         <v>340</v>
       </c>
     </row>
@@ -1863,7 +1799,7 @@
       <c r="A192" s="3" t="n">
         <v>121431</v>
       </c>
-      <c r="B192" s="0" t="n">
+      <c r="B192" s="4" t="n">
         <v>340</v>
       </c>
     </row>
@@ -1871,7 +1807,7 @@
       <c r="A193" s="3" t="n">
         <v>1271689</v>
       </c>
-      <c r="B193" s="0" t="n">
+      <c r="B193" s="4" t="n">
         <v>400</v>
       </c>
     </row>
@@ -1879,7 +1815,7 @@
       <c r="A194" s="3" t="n">
         <v>1132471</v>
       </c>
-      <c r="B194" s="0" t="n">
+      <c r="B194" s="4" t="n">
         <v>400</v>
       </c>
     </row>
@@ -1887,7 +1823,7 @@
       <c r="A195" s="3" t="n">
         <v>986117</v>
       </c>
-      <c r="B195" s="0" t="n">
+      <c r="B195" s="4" t="n">
         <v>520</v>
       </c>
     </row>
@@ -1895,7 +1831,7 @@
       <c r="A196" s="3" t="n">
         <v>986116</v>
       </c>
-      <c r="B196" s="0" t="n">
+      <c r="B196" s="4" t="n">
         <v>520</v>
       </c>
     </row>
@@ -1903,7 +1839,7 @@
       <c r="A197" s="3" t="n">
         <v>1089994</v>
       </c>
-      <c r="B197" s="0" t="n">
+      <c r="B197" s="4" t="n">
         <v>590</v>
       </c>
     </row>
@@ -1911,7 +1847,7 @@
       <c r="A198" s="3" t="n">
         <v>1089995</v>
       </c>
-      <c r="B198" s="0" t="n">
+      <c r="B198" s="4" t="n">
         <v>590</v>
       </c>
     </row>
@@ -1919,7 +1855,7 @@
       <c r="A199" s="3" t="n">
         <v>1089303</v>
       </c>
-      <c r="B199" s="0" t="n">
+      <c r="B199" s="4" t="n">
         <v>590</v>
       </c>
     </row>
@@ -1927,7 +1863,7 @@
       <c r="A200" s="3" t="n">
         <v>986600</v>
       </c>
-      <c r="B200" s="0" t="n">
+      <c r="B200" s="4" t="n">
         <v>520</v>
       </c>
     </row>
@@ -1935,7 +1871,7 @@
       <c r="A201" s="3" t="n">
         <v>986599</v>
       </c>
-      <c r="B201" s="0" t="n">
+      <c r="B201" s="4" t="n">
         <v>520</v>
       </c>
     </row>
@@ -1943,7 +1879,7 @@
       <c r="A202" s="3" t="n">
         <v>1035006</v>
       </c>
-      <c r="B202" s="0" t="n">
+      <c r="B202" s="4" t="n">
         <v>520</v>
       </c>
     </row>
@@ -1951,7 +1887,7 @@
       <c r="A203" s="3" t="n">
         <v>986598</v>
       </c>
-      <c r="B203" s="0" t="n">
+      <c r="B203" s="4" t="n">
         <v>520</v>
       </c>
     </row>
@@ -1959,7 +1895,7 @@
       <c r="A204" s="3" t="n">
         <v>986643</v>
       </c>
-      <c r="B204" s="0" t="n">
+      <c r="B204" s="4" t="n">
         <v>610</v>
       </c>
     </row>
@@ -1967,7 +1903,7 @@
       <c r="A205" s="3" t="n">
         <v>166059</v>
       </c>
-      <c r="B205" s="0" t="n">
+      <c r="B205" s="4" t="n">
         <v>610</v>
       </c>
     </row>
@@ -1975,7 +1911,7 @@
       <c r="A206" s="3" t="n">
         <v>1099402</v>
       </c>
-      <c r="B206" s="0" t="n">
+      <c r="B206" s="4" t="n">
         <v>760</v>
       </c>
     </row>

</xml_diff>